<commit_message>
Add 2026 CV PDF and update portfolio data
Add public/Alberto_Medina_CV_2026.pdf and remove the placeholder public/manifest-test.pdf. Update binary source spreadsheet src/data/content/portfolio-master.xlsx and regenerate src/data/generated/portfolioContent.json (bump generatedAt timestamp and update buttonCvHref/cvHref to "/Alberto_Medina_CV_2026.pdf") to reference the new CV.
</commit_message>
<xml_diff>
--- a/src/data/content/portfolio-master.xlsx
+++ b/src/data/content/portfolio-master.xlsx
@@ -45,7 +45,7 @@
     <t>Edit the workbook from a single control center, then sync the site.</t>
   </si>
   <si>
-    <t>MASTER WORKBOOK | LAST SYNC 2026-06-21 23:30:24 UTC | CTRL+CLICK LINKS TO NAVIGATE</t>
+    <t>MASTER WORKBOOK | LAST SYNC 2026-06-22 17:47:57 UTC | CTRL+CLICK LINKS TO NAVIGATE</t>
   </si>
   <si>
     <t>Use the cards below for primary editing, the workflow panel for the sync cycle, and the grouped panels at the bottom for advanced sheets.</t>
@@ -223,7 +223,7 @@
     <t>Editing rules, shortcuts, and the quickest path to each content area.</t>
   </si>
   <si>
-    <t>GUIDE SHEET | LAST SYNC 2026-06-21 23:30:24 UTC | START FROM HOME FOR THE FASTEST FLOW</t>
+    <t>GUIDE SHEET | LAST SYNC 2026-06-22 17:47:57 UTC | START FROM HOME FOR THE FASTEST FLOW</t>
   </si>
   <si>
     <t>Back to HOME</t>
@@ -584,7 +584,7 @@
     <t>Identity, bio headline, social links, and testimonial section copy.</t>
   </si>
   <si>
-    <t>PRIMARY EDIT SURFACE | LAST SYNC 2026-06-21 23:30:24 UTC</t>
+    <t>PRIMARY EDIT SURFACE | LAST SYNC 2026-06-22 17:47:57 UTC</t>
   </si>
   <si>
     <t>Guide</t>
@@ -740,7 +740,7 @@
     <t>CV_PENDING</t>
   </si>
   <si>
-    <t>/manifest-test.pdf</t>
+    <t>/Alberto_Medina_CV_2026.pdf</t>
   </si>
   <si>
     <t>Main project cards, value story, media wiring, and ordering.</t>
@@ -1631,7 +1631,7 @@
     <t>Brand lockup and terminal button label.</t>
   </si>
   <si>
-    <t>ADVANCED DATA SHEET | LAST SYNC 2026-06-21 23:30:24 UTC</t>
+    <t>ADVANCED DATA SHEET | LAST SYNC 2026-06-22 17:47:57 UTC</t>
   </si>
   <si>
     <t>Supporting data sheet. Changes here feed one or more primary editing surfaces.</t>

</xml_diff>